<commit_message>
Update prize categories and tracker; simplify README
Trim the dashboard and tracker to the agreed prize categories and
remove the unused display extras. Simplify the README.
</commit_message>
<xml_diff>
--- a/Tracker.xlsx
+++ b/Tracker.xlsx
@@ -23,7 +23,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -71,13 +73,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5421,7 +5424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U49"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" bestFit="1" customWidth="1" min="1" max="2"/>
@@ -5549,6 +5552,11 @@
           <t>Corners/90</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Goal Diff</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -5635,6 +5643,10 @@
         <f>IF(D2=0,0,T2/D2*90)</f>
         <v/>
       </c>
+      <c r="V2">
+        <f>E2-F2</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -5721,6 +5733,10 @@
         <f>IF(D3=0,0,T3/D3*90)</f>
         <v/>
       </c>
+      <c r="V3">
+        <f>E3-F3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -5807,6 +5823,10 @@
         <f>IF(D4=0,0,T4/D4*90)</f>
         <v/>
       </c>
+      <c r="V4">
+        <f>E4-F4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -5893,6 +5913,10 @@
         <f>IF(D5=0,0,T5/D5*90)</f>
         <v/>
       </c>
+      <c r="V5">
+        <f>E5-F5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -5979,6 +6003,10 @@
         <f>IF(D6=0,0,T6/D6*90)</f>
         <v/>
       </c>
+      <c r="V6">
+        <f>E6-F6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -6065,6 +6093,10 @@
         <f>IF(D7=0,0,T7/D7*90)</f>
         <v/>
       </c>
+      <c r="V7">
+        <f>E7-F7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -6151,6 +6183,10 @@
         <f>IF(D8=0,0,T8/D8*90)</f>
         <v/>
       </c>
+      <c r="V8">
+        <f>E8-F8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -6237,6 +6273,10 @@
         <f>IF(D9=0,0,T9/D9*90)</f>
         <v/>
       </c>
+      <c r="V9">
+        <f>E9-F9</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -6323,6 +6363,10 @@
         <f>IF(D10=0,0,T10/D10*90)</f>
         <v/>
       </c>
+      <c r="V10">
+        <f>E10-F10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -6409,6 +6453,10 @@
         <f>IF(D11=0,0,T11/D11*90)</f>
         <v/>
       </c>
+      <c r="V11">
+        <f>E11-F11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -6495,6 +6543,10 @@
         <f>IF(D12=0,0,T12/D12*90)</f>
         <v/>
       </c>
+      <c r="V12">
+        <f>E12-F12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -6581,6 +6633,10 @@
         <f>IF(D13=0,0,T13/D13*90)</f>
         <v/>
       </c>
+      <c r="V13">
+        <f>E13-F13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -6667,6 +6723,10 @@
         <f>IF(D14=0,0,T14/D14*90)</f>
         <v/>
       </c>
+      <c r="V14">
+        <f>E14-F14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -6753,6 +6813,10 @@
         <f>IF(D15=0,0,T15/D15*90)</f>
         <v/>
       </c>
+      <c r="V15">
+        <f>E15-F15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -6839,6 +6903,10 @@
         <f>IF(D16=0,0,T16/D16*90)</f>
         <v/>
       </c>
+      <c r="V16">
+        <f>E16-F16</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -6925,6 +6993,10 @@
         <f>IF(D17=0,0,T17/D17*90)</f>
         <v/>
       </c>
+      <c r="V17">
+        <f>E17-F17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -7011,6 +7083,10 @@
         <f>IF(D18=0,0,T18/D18*90)</f>
         <v/>
       </c>
+      <c r="V18">
+        <f>E18-F18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -7097,6 +7173,10 @@
         <f>IF(D19=0,0,T19/D19*90)</f>
         <v/>
       </c>
+      <c r="V19">
+        <f>E19-F19</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -7183,6 +7263,10 @@
         <f>IF(D20=0,0,T20/D20*90)</f>
         <v/>
       </c>
+      <c r="V20">
+        <f>E20-F20</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -7269,6 +7353,10 @@
         <f>IF(D21=0,0,T21/D21*90)</f>
         <v/>
       </c>
+      <c r="V21">
+        <f>E21-F21</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -7355,6 +7443,10 @@
         <f>IF(D22=0,0,T22/D22*90)</f>
         <v/>
       </c>
+      <c r="V22">
+        <f>E22-F22</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -7441,6 +7533,10 @@
         <f>IF(D23=0,0,T23/D23*90)</f>
         <v/>
       </c>
+      <c r="V23">
+        <f>E23-F23</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -7527,6 +7623,10 @@
         <f>IF(D24=0,0,T24/D24*90)</f>
         <v/>
       </c>
+      <c r="V24">
+        <f>E24-F24</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -7613,6 +7713,10 @@
         <f>IF(D25=0,0,T25/D25*90)</f>
         <v/>
       </c>
+      <c r="V25">
+        <f>E25-F25</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -7699,6 +7803,10 @@
         <f>IF(D26=0,0,T26/D26*90)</f>
         <v/>
       </c>
+      <c r="V26">
+        <f>E26-F26</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -7785,6 +7893,10 @@
         <f>IF(D27=0,0,T27/D27*90)</f>
         <v/>
       </c>
+      <c r="V27">
+        <f>E27-F27</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -7871,6 +7983,10 @@
         <f>IF(D28=0,0,T28/D28*90)</f>
         <v/>
       </c>
+      <c r="V28">
+        <f>E28-F28</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -7957,6 +8073,10 @@
         <f>IF(D29=0,0,T29/D29*90)</f>
         <v/>
       </c>
+      <c r="V29">
+        <f>E29-F29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -8043,6 +8163,10 @@
         <f>IF(D30=0,0,T30/D30*90)</f>
         <v/>
       </c>
+      <c r="V30">
+        <f>E30-F30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -8129,6 +8253,10 @@
         <f>IF(D31=0,0,T31/D31*90)</f>
         <v/>
       </c>
+      <c r="V31">
+        <f>E31-F31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -8215,6 +8343,10 @@
         <f>IF(D32=0,0,T32/D32*90)</f>
         <v/>
       </c>
+      <c r="V32">
+        <f>E32-F32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -8301,6 +8433,10 @@
         <f>IF(D33=0,0,T33/D33*90)</f>
         <v/>
       </c>
+      <c r="V33">
+        <f>E33-F33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -8387,6 +8523,10 @@
         <f>IF(D34=0,0,T34/D34*90)</f>
         <v/>
       </c>
+      <c r="V34">
+        <f>E34-F34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -8473,6 +8613,10 @@
         <f>IF(D35=0,0,T35/D35*90)</f>
         <v/>
       </c>
+      <c r="V35">
+        <f>E35-F35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -8559,6 +8703,10 @@
         <f>IF(D36=0,0,T36/D36*90)</f>
         <v/>
       </c>
+      <c r="V36">
+        <f>E36-F36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -8645,6 +8793,10 @@
         <f>IF(D37=0,0,T37/D37*90)</f>
         <v/>
       </c>
+      <c r="V37">
+        <f>E37-F37</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -8731,6 +8883,10 @@
         <f>IF(D38=0,0,T38/D38*90)</f>
         <v/>
       </c>
+      <c r="V38">
+        <f>E38-F38</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -8817,6 +8973,10 @@
         <f>IF(D39=0,0,T39/D39*90)</f>
         <v/>
       </c>
+      <c r="V39">
+        <f>E39-F39</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -8903,6 +9063,10 @@
         <f>IF(D40=0,0,T40/D40*90)</f>
         <v/>
       </c>
+      <c r="V40">
+        <f>E40-F40</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -8989,6 +9153,10 @@
         <f>IF(D41=0,0,T41/D41*90)</f>
         <v/>
       </c>
+      <c r="V41">
+        <f>E41-F41</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -9075,6 +9243,10 @@
         <f>IF(D42=0,0,T42/D42*90)</f>
         <v/>
       </c>
+      <c r="V42">
+        <f>E42-F42</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -9161,6 +9333,10 @@
         <f>IF(D43=0,0,T43/D43*90)</f>
         <v/>
       </c>
+      <c r="V43">
+        <f>E43-F43</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -9247,6 +9423,10 @@
         <f>IF(D44=0,0,T44/D44*90)</f>
         <v/>
       </c>
+      <c r="V44">
+        <f>E44-F44</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -9333,6 +9513,10 @@
         <f>IF(D45=0,0,T45/D45*90)</f>
         <v/>
       </c>
+      <c r="V45">
+        <f>E45-F45</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -9419,6 +9603,10 @@
         <f>IF(D46=0,0,T46/D46*90)</f>
         <v/>
       </c>
+      <c r="V46">
+        <f>E46-F46</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -9505,6 +9693,10 @@
         <f>IF(D47=0,0,T47/D47*90)</f>
         <v/>
       </c>
+      <c r="V47">
+        <f>E47-F47</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -9591,6 +9783,10 @@
         <f>IF(D48=0,0,T48/D48*90)</f>
         <v/>
       </c>
+      <c r="V48">
+        <f>E48-F48</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -9675,6 +9871,10 @@
       </c>
       <c r="U49" s="3">
         <f>IF(D49=0,0,T49/D49*90)</f>
+        <v/>
+      </c>
+      <c r="V49">
+        <f>E49-F49</f>
         <v/>
       </c>
     </row>
@@ -9689,7 +9889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9718,6 +9918,11 @@
           <t>Value</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Prize (£)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9737,15 +9942,18 @@
         <f>MAX('Team Totals'!$H$2:$H$49)</f>
         <v/>
       </c>
+      <c r="E2" s="6" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Most Shots on Target / 90</t>
+          <t>Highest Avg Possession %</t>
         </is>
       </c>
       <c r="B3">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$J$2:$J$49),'Team Totals'!$J$2:$J$49,0)),"")</f>
+        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$K$2:$K$49),'Team Totals'!$K$2:$K$49,0)),"")</f>
         <v/>
       </c>
       <c r="C3">
@@ -9753,18 +9961,21 @@
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>MAX('Team Totals'!$J$2:$J$49)</f>
-        <v/>
+        <f>MAX('Team Totals'!$K$2:$K$49)</f>
+        <v/>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Highest Avg Possession %</t>
+          <t>Most Fouls / 90</t>
         </is>
       </c>
       <c r="B4">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$K$2:$K$49),'Team Totals'!$K$2:$K$49,0)),"")</f>
+        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$M$2:$M$49),'Team Totals'!$M$2:$M$49,0)),"")</f>
         <v/>
       </c>
       <c r="C4">
@@ -9772,18 +9983,21 @@
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>MAX('Team Totals'!$K$2:$K$49)</f>
-        <v/>
+        <f>MAX('Team Totals'!$M$2:$M$49)</f>
+        <v/>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Most Fouls / 90</t>
+          <t>Most Offsides / 90</t>
         </is>
       </c>
       <c r="B5">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$M$2:$M$49),'Team Totals'!$M$2:$M$49,0)),"")</f>
+        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$S$2:$S$49),'Team Totals'!$S$2:$S$49,0)),"")</f>
         <v/>
       </c>
       <c r="C5">
@@ -9791,18 +10005,21 @@
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>MAX('Team Totals'!$M$2:$M$49)</f>
-        <v/>
+        <f>MAX('Team Totals'!$S$2:$S$49)</f>
+        <v/>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Most Cards / 90 (Y=1, R=2)</t>
+          <t>Most Corners / 90</t>
         </is>
       </c>
       <c r="B6">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$Q$2:$Q$49),'Team Totals'!$Q$2:$Q$49,0)),"")</f>
+        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$U$2:$U$49),'Team Totals'!$U$2:$U$49,0)),"")</f>
         <v/>
       </c>
       <c r="C6">
@@ -9810,18 +10027,21 @@
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>MAX('Team Totals'!$Q$2:$Q$49)</f>
-        <v/>
+        <f>MAX('Team Totals'!$U$2:$U$49)</f>
+        <v/>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Most Offsides / 90</t>
+          <t>Largest Negative Goal Difference</t>
         </is>
       </c>
       <c r="B7">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$S$2:$S$49),'Team Totals'!$S$2:$S$49,0)),"")</f>
+        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MIN('Team Totals'!$V$2:$V$49),'Team Totals'!$V$2:$V$49,0)),"")</f>
         <v/>
       </c>
       <c r="C7">
@@ -9829,48 +10049,17 @@
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>MAX('Team Totals'!$S$2:$S$49)</f>
-        <v/>
+        <f>MIN('Team Totals'!$V$2:$V$49)</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Most Corners / 90</t>
-        </is>
-      </c>
-      <c r="B8">
-        <f>IFERROR(INDEX('Team Totals'!$A$2:$A$49,MATCH(MAX('Team Totals'!$U$2:$U$49),'Team Totals'!$U$2:$U$49,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>IFERROR(VLOOKUP(B8,Participants!$B$2:$C$49,2,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="D8" s="3">
-        <f>MAX('Team Totals'!$U$2:$U$49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Largest Goal Difference (single match)</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>IFERROR(INDEX('Match Data'!$Y$2:$Y$201,MATCH(MAX('Match Data'!$X$2:$X$201),'Match Data'!$X$2:$X$201,0)),"")</f>
-        <v/>
-      </c>
-      <c r="C9">
-        <f>IFERROR(VLOOKUP(B9,Participants!$B$2:$C$49,2,FALSE),"")</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>IFERROR(MAX('Match Data'!$X$2:$X$201),0)</f>
-        <v/>
-      </c>
-    </row>
+      <c r="D8" s="3" t="n"/>
+    </row>
+    <row r="9"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9882,7 +10071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9911,6 +10100,11 @@
           <t>Entrant</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Prize (£)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -9922,6 +10116,9 @@
         <f>IFERROR(VLOOKUP(C2,Participants!$B$2:$C$49,2,FALSE),"")</f>
         <v/>
       </c>
+      <c r="E2" s="6" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -9933,6 +10130,9 @@
         <f>IFERROR(VLOOKUP(C3,Participants!$B$2:$C$49,2,FALSE),"")</f>
         <v/>
       </c>
+      <c r="E3" s="6" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -9944,6 +10144,9 @@
         <f>IFERROR(VLOOKUP(C4,Participants!$B$2:$C$49,2,FALSE),"")</f>
         <v/>
       </c>
+      <c r="E4" s="6" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -9952,8 +10155,11 @@
         </is>
       </c>
       <c r="D5">
-        <f>IFERROR(VLOOKUP(C6,Participants!$B$2:$C$49,2,FALSE),"")</f>
-        <v/>
+        <f>IFERROR(VLOOKUP(C5,Participants!$B$2:$C$49,2,FALSE),"")</f>
+        <v/>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>